<commit_message>
Fix import test cases to validate for each validation mode
Alter rdi file
</commit_message>
<xml_diff>
--- a/tests/data/rdi_with_references.xlsx
+++ b/tests/data/rdi_with_references.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,7 +13,7 @@
     <sheet name="People" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$A$1:$Q$11</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$A$1:$P$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="120">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -48,18 +48,9 @@
     <t xml:space="preserve">size_h_c</t>
   </si>
   <si>
-    <t xml:space="preserve">hh_latrine_h_f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hh_electricity_h_f</t>
-  </si>
-  <si>
     <t xml:space="preserve">registration_method_h_c</t>
   </si>
   <si>
-    <t xml:space="preserve">collect_individual_data_h_c</t>
-  </si>
-  <si>
     <t xml:space="preserve">name_enumerator_h_c</t>
   </si>
   <si>
@@ -69,9 +60,6 @@
     <t xml:space="preserve">consent_sharing_h_c</t>
   </si>
   <si>
-    <t xml:space="preserve">first_registration_date_h_c</t>
-  </si>
-  <si>
     <t xml:space="preserve">head_of_household_id</t>
   </si>
   <si>
@@ -150,13 +138,10 @@
     <t xml:space="preserve">phone_no_i_c</t>
   </si>
   <si>
-    <t xml:space="preserve">first_registration_date_i_c</t>
-  </si>
-  <si>
     <t xml:space="preserve">disability_i_c</t>
   </si>
   <si>
-    <t xml:space="preserve">HEAD</t>
+    <t xml:space="preserve">MOTHER_FATHER</t>
   </si>
   <si>
     <t xml:space="preserve">Edward Jeffrey Rogers</t>
@@ -506,7 +491,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -521,6 +506,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -599,9 +588,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>726840</xdr:colOff>
+      <xdr:colOff>726120</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>108000</xdr:rowOff>
+      <xdr:rowOff>107280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -615,7 +604,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17568720" y="2095560"/>
-          <a:ext cx="726840" cy="298440"/>
+          <a:ext cx="726120" cy="297720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -637,9 +626,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>96120</xdr:colOff>
+      <xdr:colOff>95400</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93240</xdr:rowOff>
+      <xdr:rowOff>92520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -653,7 +642,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10992960" y="380880"/>
-          <a:ext cx="96120" cy="93240"/>
+          <a:ext cx="95400" cy="92520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -675,9 +664,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>96120</xdr:colOff>
+      <xdr:colOff>95400</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93240</xdr:rowOff>
+      <xdr:rowOff>92520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -691,7 +680,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17568720" y="380880"/>
-          <a:ext cx="96120" cy="93240"/>
+          <a:ext cx="95400" cy="92520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -718,9 +707,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>95760</xdr:colOff>
+      <xdr:colOff>95040</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93240</xdr:rowOff>
+      <xdr:rowOff>92520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -734,7 +723,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5689440" y="454680"/>
-          <a:ext cx="95760" cy="93240"/>
+          <a:ext cx="95040" cy="92520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -930,7 +919,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R1048576"/>
+  <dimension ref="A1:N1048576"/>
   <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.34"/>
@@ -938,16 +927,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="11.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="10.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="24.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="33.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="46.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="29.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="33.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="46.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="29.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -992,18 +979,6 @@
       </c>
       <c r="N1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1014,12 +989,10 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -1030,51 +1003,39 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="P3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="1" t="n">
+      <c r="M3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="R3" s="1" t="n">
+      <c r="N3" s="1" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1087,51 +1048,39 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>1</v>
+      <c r="H4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="P4" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="Q4" s="1" t="n">
+      <c r="M4" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="R4" s="1" t="n">
+      <c r="N4" s="1" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1157,7 +1106,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q1048576"/>
+  <dimension ref="A1:P1048576"/>
   <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.5"/>
@@ -1174,9 +1123,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="11.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="11.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1184,52 +1132,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1249,7 +1194,6 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -1258,45 +1202,42 @@
       <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="5" t="n">
         <v>28558</v>
       </c>
       <c r="K3" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="P3" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>51</v>
+      <c r="L3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1307,35 +1248,32 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>24971</v>
       </c>
       <c r="K4" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>56</v>
+      <c r="P4" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1346,45 +1284,42 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>24092</v>
       </c>
       <c r="K5" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M5" s="5" t="e">
+      <c r="L5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="6" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>56</v>
+      <c r="N5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1395,45 +1330,42 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J6" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>43298</v>
       </c>
       <c r="K6" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="M6" s="5" t="e">
+      <c r="L6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="6" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>56</v>
+      <c r="N6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1444,35 +1376,32 @@
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="J7" s="5" t="n">
         <v>34615</v>
       </c>
       <c r="K7" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P7" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q7" s="5" t="s">
-        <v>56</v>
+      <c r="P7" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1483,35 +1412,32 @@
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="J8" s="5" t="n">
         <v>25778</v>
       </c>
       <c r="K8" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>51</v>
+      <c r="P8" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,35 +1448,32 @@
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J9" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="J9" s="5" t="n">
         <v>31934</v>
       </c>
       <c r="K9" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P9" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>56</v>
+      <c r="P9" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1560,45 +1483,42 @@
       <c r="B10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" s="4" t="n">
+      <c r="J10" s="5" t="n">
         <v>23346</v>
       </c>
       <c r="K10" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>45095</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>56</v>
+      <c r="L10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1609,33 +1529,30 @@
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D11" s="1" t="str">
         <f aca="false">E11&amp;" "&amp;F11&amp;" "&amp;G11</f>
         <v>Nataly Catherine Douglas</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J11" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="J11" s="5" t="n">
         <v>42889</v>
       </c>
       <c r="K11" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
-      </c>
-      <c r="P11" s="4" t="n">
-        <v>45095</v>
       </c>
     </row>
     <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1661,7 +1578,7 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:Q11"/>
+  <autoFilter ref="A1:P11"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1682,251 +1599,251 @@
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="I1" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="J1" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="K1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="M1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="O1" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="Q1" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="R1" s="7" t="s">
         <v>99</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+      <c r="A2" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>37125</v>
+      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="L2" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" s="11" t="n">
-        <v>37125</v>
-      </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="12" t="s">
+      <c r="N2" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="R2" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" s="11" t="n">
+      <c r="B3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="10"/>
+      <c r="E3" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="12" t="n">
         <v>40777</v>
       </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="12" t="s">
+      <c r="H3" s="8"/>
+      <c r="I3" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="N3" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="R3" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="N3" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" s="11" t="n">
+      <c r="B4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="10"/>
+      <c r="E4" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="12" t="n">
         <v>33472</v>
       </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="12" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="N4" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="R4" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="N4" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="R4" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" s="11" t="n">
+      <c r="B5" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="12" t="n">
         <v>36760</v>
       </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="12" t="s">
+      <c r="H5" s="8"/>
+      <c r="I5" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="N5" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="R5" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="N5" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="R5" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new test cases for validation modes when importing people
Alter rdi_with_references.xlsx file
</commit_message>
<xml_diff>
--- a/tests/data/rdi_with_references.xlsx
+++ b/tests/data/rdi_with_references.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="104">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -298,33 +298,6 @@
   </si>
   <si>
     <t xml:space="preserve">pp_address_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_country_origin_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_country_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_zip_code_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_admin1_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_admin2_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_admin3_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_admin4_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_residence_status_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pp_consent_i_c</t>
   </si>
   <si>
     <t xml:space="preserve">Collector ForJanIndex_3</t>
@@ -338,27 +311,6 @@
   <si>
     <t xml:space="preserve">938 Luna Cliffs Apt. 551
 Jameschester, SC 24934</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AF11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AF1115</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFUGEE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRUE</t>
   </si>
   <si>
     <t xml:space="preserve">WorkerCollector ForDerekIndex_4</t>
@@ -491,7 +443,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -508,15 +460,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -588,9 +536,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>726120</xdr:colOff>
+      <xdr:colOff>725400</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>107280</xdr:rowOff>
+      <xdr:rowOff>106560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -604,7 +552,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17568720" y="2095560"/>
-          <a:ext cx="726120" cy="297720"/>
+          <a:ext cx="725400" cy="297000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -626,9 +574,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>95400</xdr:colOff>
+      <xdr:colOff>94680</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>92520</xdr:rowOff>
+      <xdr:rowOff>91800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -642,7 +590,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10992960" y="380880"/>
-          <a:ext cx="95400" cy="92520"/>
+          <a:ext cx="94680" cy="91800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -664,9 +612,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>95400</xdr:colOff>
+      <xdr:colOff>94680</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>92520</xdr:rowOff>
+      <xdr:rowOff>91800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -680,7 +628,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17568720" y="380880"/>
-          <a:ext cx="95400" cy="92520"/>
+          <a:ext cx="94680" cy="91800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -707,9 +655,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>95040</xdr:colOff>
+      <xdr:colOff>94320</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>92520</xdr:rowOff>
+      <xdr:rowOff>91800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -722,8 +670,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5689440" y="454680"/>
-          <a:ext cx="95040" cy="92520"/>
+          <a:off x="5798160" y="454680"/>
+          <a:ext cx="94320" cy="91800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1227,16 +1175,16 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="4" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1272,7 +1220,7 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="P4" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1308,17 +1256,17 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="L5" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="6" t="e">
+      <c r="M5" s="4" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P5" s="6" t="s">
+      <c r="P5" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1354,17 +1302,17 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="L6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="6" t="e">
+      <c r="M6" s="4" t="e">
         <f aca="false">#VALUE!</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="6" t="s">
+      <c r="P6" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1400,7 +1348,7 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="P7" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1436,7 +1384,7 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" s="4" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1472,7 +1420,7 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="P9" s="6" t="s">
+      <c r="P9" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1508,16 +1456,16 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O10" s="6" t="s">
+      <c r="O10" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="P10" s="6" t="s">
+      <c r="P10" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1595,255 +1543,140 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.02"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q1" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="R1" s="7" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="n">
+      <c r="A2" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" s="11" t="s">
+      <c r="B2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="12" t="n">
+      <c r="G2" s="11" t="n">
         <v>37125</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>110</v>
+      <c r="H2" s="7"/>
+      <c r="I2" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="F3" s="11" t="s">
+      <c r="B3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="G3" s="11" t="n">
         <v>40777</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>110</v>
+      <c r="H3" s="7"/>
+      <c r="I3" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="F4" s="11" t="s">
+      <c r="B4" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="11" t="n">
         <v>33472</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="R4" s="7" t="s">
-        <v>110</v>
+      <c r="H4" s="7"/>
+      <c r="I4" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" s="11" t="s">
+      <c r="B5" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="11" t="n">
         <v>36760</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>110</v>
+      <c r="H5" s="7"/>
+      <c r="I5" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>